<commit_message>
Stage 8 fixes: B-026
</commit_message>
<xml_diff>
--- a/output/archive/BrindlewytheData/Studies/2025/BW25_0600/Run_sheets/BW25_0600_RUN04.xlsx
+++ b/output/archive/BrindlewytheData/Studies/2025/BW25_0600/Run_sheets/BW25_0600_RUN04.xlsx
@@ -738,7 +738,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:H34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -806,7 +806,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>AP02-01400 to 01412</t>
+          <t>Interim primary-assay plate map in compound sample cards under B-ACC-2025-10218</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -848,7 +848,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>AP02-01414 to 01424</t>
+          <t>Remaining interim primary-assay assignments in the same compound sample-card register; no contiguous ID block assumed</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -977,6 +977,431 @@
       <c r="A9" s="1" t="inlineStr">
         <is>
           <t>Plate acceptance: all four plates accepted for the final fit and the sweep.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Compound</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Auditable sample-card reference</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>Plate / replicate source</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01400</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01400 sample card</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01410</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01410 sample card</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01416</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01416 sample card</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01418</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01418 sample card</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01428</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01428 sample card</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01430</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01430 sample card</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01440</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01440 sample card</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01446</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01446 sample card</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01452</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01452 sample card</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01458</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01458 sample card</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01460</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01460 sample card</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01466</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01466 sample card</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01470</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01470 sample card</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01488</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01488 sample card</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01494</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01494 sample card</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01502</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01502 sample card</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01506</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01506 sample card</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01508</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01508 sample card</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01518</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01518 sample card</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01536</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01536 sample card</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01574</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01574 sample card</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01580</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01580 sample card</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01584</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01584 sample card</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>AP02-01590</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>B-ACC-2025-10218: AP02-01590 sample card</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>Interim plate/well map and final repeat run/fit record retained with this card</t>
         </is>
       </c>
     </row>
@@ -1015,7 +1440,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Hill slopes outside the study plan window were re-fitted with the top fixed before the value was accepted. Replicate fits are on the run sheet.</t>
+          <t>Out-of-window Hill slopes were reviewed under the study plan and rerun or excluded as appropriate. Replicate measurements and fit dispositions remain in the compound-linked primary-assay run records under B-ACC-2025-10218, referenced by the Plate acceptance sample-card register; this sheet contains accepted summaries only. A constrained top requires a documented control-supported plateau and reviewer rationale in that fit record; fixing the top alone does not establish acceptance.</t>
         </is>
       </c>
     </row>

</xml_diff>